<commit_message>
Update favalli experiment: lane-1-fasta -> lane-1 paths throughout
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/supporting_material/experiments/favalli/lane-1.xlsx
+++ b/supporting_material/experiments/favalli/lane-1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10525"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adrianomartinelli/projects/delt-hit/supporting_material/experiments/favalli/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0DC5562-F08A-7B46-A5CA-60D6E33F0D28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{289A6224-7518-EA41-B502-15E72A528C80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15120" yWindow="660" windowWidth="15120" windowHeight="18980" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="15120" yWindow="660" windowWidth="15120" windowHeight="18980" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="experiment" sheetId="8" r:id="rId1"/>
@@ -4591,7 +4591,7 @@
     <t>./20190812.A-1907_NF2GB2_s1_R1.fasta.gz</t>
   </si>
   <si>
-    <t>lane-1-fasta</t>
+    <t>lane-1</t>
   </si>
 </sst>
 </file>

</xml_diff>